<commit_message>
feat(obsidian): synchronize all docs reference integrity audit outputs to pass CI
</commit_message>
<xml_diff>
--- a/mighty-link-ai-connect.xlsx
+++ b/mighty-link-ai-connect.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\mighty-link-ai-connect\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B71CE880-4F7A-4B64-8469-876820648532}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4AB063C-92A5-4AEF-9237-3EA99774800A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{66EF4EAD-7CE3-414D-A20B-206D64169BF2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{66EF4EAD-7CE3-414D-A20B-206D64169BF2}"/>
   </bookViews>
   <sheets>
     <sheet name="ソースコードレビュー" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="39">
   <si>
     <t>C:\Users\kanta\GitHub\mighty-link-ai-connect\__pycache__</t>
     <phoneticPr fontId="1"/>
@@ -1992,1041 +1992,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Segoe UI Symbol"/>
-        <family val="2"/>
-      </rPr>
-      <t>📁</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> __pycache__ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>フォルダの概要と解説</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-1. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>概要と役割</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-__pycache__ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>は、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Python </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>インタプリタ（この環境では</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> Python 3.12</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>）がソースコード（</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>.py</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>）を実行・インポートする際に自動生成するコンパイル済みバイトコード（</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>.pyc</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>）を格納するキャッシュフォルダです。</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>目的</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>次回の実行時に</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> Python </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>ソースコードの構文解析（コンパイル）処理を省き、モジュールの読み込み速度・起動スピードを向上させるために機能します。</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>自動管理</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>ソースコード（</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>.py</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>）が更新されると、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Python </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>がタイムスタンプを検知して自動的に最新の</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> .pyc </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>ファイルへ再生成します。</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-2. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>現在のフォルダー内容</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>現在、このフォルダ内には以下のファイルが格納されています：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-main.cpython-312.pyc
- (</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>サイズ</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>約</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> 3.3 KB)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>プロジェクト直下の</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> 
-main.py
- </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>を</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> Python 3.12 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>環境で実行・インポートした際に生成されたバイトコードキャッシュです。</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Segoe UI Symbol"/>
-        <family val="2"/>
-      </rPr>
-      <t>🔍</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>コードレビュー・運用評価</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>評価項目</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">	</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>判定</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">	</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>評価内容</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Git </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>バージョン管理</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">	</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Segoe UI Symbol"/>
-        <family val="2"/>
-      </rPr>
-      <t>✅</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>適正</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">	
- .gitignore
- </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>の</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> 7</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>〜</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">8 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>行目に</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> __pycache__/ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>および</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> *.pyc </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>が登録されており、リポジトリへ無駄なバイナリがコミットされないよう適切に保護されています。</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>セキュリティ・機密性</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">	</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Segoe UI Symbol"/>
-        <family val="2"/>
-      </rPr>
-      <t>✅</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>適正</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">	.pyc </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>ファイルは簡単な逆コンパイルが可能ですが、参照元の</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> main.py </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>内にハードコードされた秘密鍵やトークンは存在せず環境変数化されているため、キャッシュからの情報漏洩リスクもありません。</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>ファイル構成の健全性</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">	</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Segoe UI Symbol"/>
-        <family val="2"/>
-      </rPr>
-      <t>✅</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>健全</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">	</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>キャッシュの蓄積や肥大化はなく、最新の起動結果のみが保持されています。</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Segoe UI Symbol"/>
-        <family val="2"/>
-      </rPr>
-      <t>💡</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>運用上の注意点・メンテナンス</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-__pycache__ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>フォルダは一時的に削除しても、次回</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> Python </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>実行時に自動生成されるため安全に削除可能です。</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>キャッシュを強制クリアしたい場合は、以下のコマンド等で一括削除できます：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-powershell
-# PowerShell </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="游ゴシック"/>
-        <family val="2"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>でのキャッシュクリア例</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Get-ChildItem -Path . -Recurse -Filter "__pycache__" | Remove-Item -Recurse -Force</t>
-    </r>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>C:\Users\kanta\GitHub\mighty-link-ai-connect\backups</t>
     <phoneticPr fontId="1"/>
   </si>
@@ -9258,6 +8223,2958 @@
   </si>
   <si>
     <t>C:\Users\kanta\GitHub\mighty-link-ai-connect\db</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>📁</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">db/ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>フォルダの概要と解説</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+1. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>概要と目的</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+db/ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>フォルダは、本アプリケーションのランタイム・データベーススキーマのマイグレーション（テーブル定義変更履歴・</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>DDL SQL</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）を管理するディレクトリです。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>マイグレーション実行スクリプト</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> 
+scripts/manage_db_migrations.py
+ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>と連携し、ローカル開発・テスト用の</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> SQLite </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>と本番・</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>UAT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>用の</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Supabase / PostgreSQL </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>の双方でスキーマの整合性を保ちながらバージョン管理を行っています。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+2. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ディレクトリ構成と主要ファイル</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>📄</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">A. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ガイドライン</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (
+db/migrations/README.md
+)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>マイグレーション運用のルールが厳格に定義されています：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>イミュータブル運用</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>共有</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> DB </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>に適用済みのマイグレーションは変更せず、修正時は新たな前進マイグレーション（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Forward-fix</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）を追加する。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>命名規約</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>: YYYYMMDDHHMMSS_short_slug.sql (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>例</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: 20260618000000_sales_email_matching_schema.sql)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>事前検証</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>コミット前に</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> python scripts/manage_db_migrations.py validate </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>および</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> --dry-run </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>で動作を事前確認する。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Emoji"/>
+        <family val="2"/>
+      </rPr>
+      <t>🗄️</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">B. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>マイグレーションスクリプト</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (db/migrations/)
+sqlite/
+: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ローカル</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> SQLite (data/mighty.db </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>やテスト環境</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> data_test/) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>向け</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> DDL </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>スクリプト。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+20260614000000_app_core_schema.sql (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>コアテーブル</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>: engineers, jobs, matches)
+20260616000000_feedback_events.sql (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>フィードバックログ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>)
+20260616000001_support_requests.sql (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>問い合わせ管理</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>)
+20260618000000_sales_email_matching_schema.sql (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>営業メールパース・マッチングテーブル</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">)
+postgres/
+: Supabase / PostgreSQL </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>方言に適合した同一バージョン・同等構造の</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> DDL </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>スクリプト。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+rollback/
+: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>万が一の本番障害時やスキーマ巻き戻し用の切り戻し用</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> SQL </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>スクリプト。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+3. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>他のマイグレーションフォルダとの役割分担</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>本プロジェクトでは</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> DB </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>定義が</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> 2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>つのフォルダで役割分担されています：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>フォルダ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">	</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>主な対象と管理内容</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+db/migrations/ (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>本フォルダ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">)	</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>アプリケーション層テーブル</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: FastAPI / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>スクリプトから直接</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> CRUD </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>される業務テーブル群。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+supabase/migrations/	</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>インフラ・セキュリティ層</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: Supabase CLI </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>により管理される</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> RLS (Row Level Security) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ポリシー、認証</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (Auth)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">pgvector </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>拡張など。</t>
+    </r>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>🔍</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>コードレビュー・運用評価</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>評価項目</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">	</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>判定</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">	</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>評価内容</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>スキーマ漂流の防止</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (Schema Drift Protection)	</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>✅</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>極めて優良</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">	</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>同一のバージョン番号で</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> sqlite/ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>と</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> postgres/ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>の両</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> DDL </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>が保持されており、ローカルテスト環境と本番環境でのスキーマ乖離が発生しない設計です。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>運用ガバナンス・安全性</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">	</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>✅</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>優良</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">	README.md </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>にて適用済みファイルの変更禁止や</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> --dry-run </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>必須化がルール化され、管理スクリプト</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> manage_db_migrations.py </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>でコマンド自動化されています。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ロールバック（切り戻し）対応</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">	</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>✅</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>優良</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">	rollback/ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ディレクトリに削除・復旧用</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> SQL </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>スクリプトを用意しておくことで、リリース時のダウンタイムや障害発生のリスクが最小化されています。</t>
+    </r>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>📁</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> __pycache__ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>フォルダの概要と解説</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+1. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>概要と役割</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+__pycache__ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>は、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Python </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>インタプリタ（この環境では</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Python 3.12</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）がソースコード（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>.py</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）を実行・インポートする際に自動生成するコンパイル済みバイトコード（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>.pyc</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）を格納するキャッシュフォルダです。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>目的</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>次回の実行時に</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Python </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ソースコードの構文解析（コンパイル）処理を省き、モジュールの読み込み速度・起動スピードを向上させるために機能します。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>自動管理</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ソースコード（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>.py</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）が更新されると、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Python </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>がタイムスタンプを検知して自動的に最新の</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> .pyc </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ファイルへ再生成します。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+2. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>現在のフォルダー内容</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>現在、このフォルダ内には以下のファイルが格納されています：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+main.cpython-312.pyc
+ (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>サイズ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>約</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> 3.3 KB)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>プロジェクト直下の</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> 
+main.py
+ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>を</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Python 3.12 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>環境で実行・インポートした際に生成されたバイトコードキャッシュです。</t>
+    </r>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>🔍</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>コードレビュー・運用評価</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>評価項目</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">	</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>判定</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">	</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>評価内容</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Git </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>バージョン管理</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">	</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>✅</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>適正</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">	
+ .gitignore
+ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>の</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> 7</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>〜</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">8 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>行目に</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> __pycache__/ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>および</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> *.pyc </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>が登録されており、リポジトリへ無駄なバイナリがコミットされないよう適切に保護されています。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>セキュリティ・機密性</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">	</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>✅</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>適正</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">	.pyc </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ファイルは簡単な逆コンパイルが可能ですが、参照元の</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> main.py </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>内にハードコードされた秘密鍵やトークンは存在せず環境変数化されているため、キャッシュからの情報漏洩リスクもありません。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ファイル構成の健全性</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">	</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>✅</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>健全</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">	</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>キャッシュの蓄積や肥大化はなく、最新の起動結果のみが保持されています。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>💡</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>運用上の注意点・メンテナンス</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+__pycache__ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>フォルダは一時的に削除しても、次回</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Python </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>実行時に自動生成されるため安全に削除可能です。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>キャッシュを強制クリアしたい場合は、以下のコマンド等で一括削除できます：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+powershell
+# PowerShell </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>でのキャッシュクリア例</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Get-ChildItem -Path . -Recurse -Filter "__pycache__" | Remove-Item -Recurse -Force</t>
+    </r>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>例外処理</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Emoji"/>
+        <family val="2"/>
+      </rPr>
+      <t>⚠️</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 「例外処理（Exception Handling）」の解説
+例外処理とは、**「プログラムの実行中に発生する予期しないエラー（DB接続断、ネットワークタイムアウト、ファイル不整合、不正なユーザー入力など）を捕捉（catch / except）し、プログラムの強制終了（クラッシュ）を防いで安全にエラー制御・回復・通知を行うプログラミング構造および設計方針」**を指します。
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>💡</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>本プロジェクト（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mighty Skill-Bridge</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）における主な例外処理方針と品質ルール</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>エラー握りつぶし・無症状パッチの厳禁</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">:
+try-except </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>でエラーを無視して空のデータを返したり、サイレントに飲み込む修正（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Superficial Symptom Patches</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）を明確に禁止。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Fail-closed </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>原則の徹底</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>認証失敗や予期せぬ例外が発生した場合、データを漏洩させず即座に安全側（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>503/401/403</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>遮断）へ倒す。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>自動監査ガードによる網羅検証</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>フォームや</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>UI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>のエラーハンドリング（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>audit_form_error_handling.py</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>管理画面のエラーハンドリング（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>audit_admin_dashboard_error_handling.py</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>診断フォールバックの透明性（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>audit_diagnosis_fallback_transparency.py</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）</t>
+    </r>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -9692,7 +11609,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="2:7" ht="409.5" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:7" ht="281.25" x14ac:dyDescent="0.4">
       <c r="B3" t="s">
         <v>1</v>
       </c>
@@ -9702,8 +11619,11 @@
       <c r="D3" t="s">
         <v>0</v>
       </c>
+      <c r="E3" s="1" t="s">
+        <v>36</v>
+      </c>
       <c r="F3" s="1" t="s">
-        <v>14</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="2:7" ht="409.5" x14ac:dyDescent="0.4">
@@ -9736,13 +11656,13 @@
         <v>3</v>
       </c>
       <c r="D5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="2:7" ht="409.5" x14ac:dyDescent="0.4">
@@ -9754,14 +11674,15 @@
         <v>4</v>
       </c>
       <c r="D6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>26</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
+      <c r="G6" s="1"/>
     </row>
     <row r="7" spans="2:7" ht="409.5" x14ac:dyDescent="0.4">
       <c r="C7">
@@ -9769,21 +11690,28 @@
         <v>5</v>
       </c>
       <c r="D7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>29</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
+      <c r="G7" s="1"/>
     </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.4">
+    <row r="8" spans="2:7" ht="409.5" x14ac:dyDescent="0.4">
       <c r="C8">
         <f>C7+1</f>
         <v>6</v>
       </c>
       <c r="D8" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -9795,7 +11723,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D61D7BD1-E21E-491C-9734-845F33AEBE13}">
-  <dimension ref="B3:E9"/>
+  <dimension ref="B3:E10"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="3.375" bestFit="1" customWidth="1"/>
@@ -9845,7 +11773,7 @@
         <v>6</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="2:5" ht="202.5" x14ac:dyDescent="0.4">
@@ -9857,10 +11785,10 @@
         <v>4</v>
       </c>
       <c r="D6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="2:5" ht="292.5" x14ac:dyDescent="0.4">
@@ -9872,10 +11800,10 @@
         <v>5</v>
       </c>
       <c r="D7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="2:5" ht="258.75" x14ac:dyDescent="0.4">
@@ -9887,10 +11815,10 @@
         <v>6</v>
       </c>
       <c r="D8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="2:5" ht="277.5" x14ac:dyDescent="0.4">
@@ -9902,10 +11830,25 @@
         <v>7</v>
       </c>
       <c r="D9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" ht="281.25" x14ac:dyDescent="0.4">
+      <c r="B10" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10">
+        <f>C9+1</f>
+        <v>8</v>
+      </c>
+      <c r="D10" t="s">
+        <v>37</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(wbs): sync WBS.md, Google Calendar, and Knowledge Graph (387 tasks)
</commit_message>
<xml_diff>
--- a/mighty-link-ai-connect.xlsx
+++ b/mighty-link-ai-connect.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\mighty-link-ai-connect\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56E25A36-5D92-4B62-A261-C0D9A14BD155}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98FA7342-29EE-4183-AAF1-2A777D3FA3E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{66EF4EAD-7CE3-414D-A20B-206D64169BF2}"/>
   </bookViews>
   <sheets>
     <sheet name="ソースコードレビュー" sheetId="1" r:id="rId1"/>
     <sheet name="用語集" sheetId="2" r:id="rId2"/>
-    <sheet name="YouTube" sheetId="3" r:id="rId3"/>
-    <sheet name="ブログ" sheetId="4" r:id="rId4"/>
+    <sheet name="OpenAIAcademy" sheetId="5" r:id="rId3"/>
+    <sheet name="YouTube" sheetId="3" r:id="rId4"/>
+    <sheet name="ブログ" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="86">
   <si>
     <t>C:\Users\kanta\GitHub\mighty-link-ai-connect\__pycache__</t>
     <phoneticPr fontId="1"/>
@@ -16025,6 +16026,3220 @@
         <scheme val="minor"/>
       </rPr>
       <t>障害・セキュリティ事案発生時のタイムライン特定および原因究明プロセス。</t>
+    </r>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>RAG</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://academy.openai.com/learn/ai-foundations-juzjs/lessons</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>🔍</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>「</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>RAG</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Retrieval-Augmented Generation / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>検索拡張生成）」の解説</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+**RAG</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（検索拡張生成）とは、「</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>LLM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（大規模言語モデル）の持つ高い自然言語生成能力と、外部のデータベース・ナレッジベースからの高度な情報検索（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Retrieval</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）機構を組み合わせるアーキテクチャ」</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>**</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>を指します。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+LLM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>単体で発生しやすい</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>**</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ハルシネーション（事実と異なる事実誤認や嘘の回答の生成）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>**</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>を劇的に抑え、社内独自のドキュメントやリアルタイム・最新の情報をコンテキストとして注入することで、信頼性の高い正確な回答を提示できます。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>💡</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> RAG</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>の基本プロセス（処理フロー）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>インデックス化（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Indexing</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>社内文書・ナレッジ（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Markdown, PDF</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>等）を短文ブロック（チャンク）に分割し、ベクトルエンベディングに変換してベクトルストアへ蓄積。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>関連情報検索（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Retrieval</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ユーザーからの質問文をベクトル化し、意味的に最も関連性の高い文書チャンクを上位検索・抽出。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>回答生成（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Generation</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>抽出した関連文書をプロンプト文脈（コンテキスト）として</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>LLM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Gemini</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>等）に提示し、根拠のある回答を構成。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>💡</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>本プロダクト（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mighty Skill-Bridge</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）での主な活用場所</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>営業メール</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>マッチング</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>人材データベースや案件要求要件の検索文脈を抽出し、適合度スコアリングと根拠テキストの自動抽出に活用。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+NotebookLM &amp; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ナレッジ同期パイプライン</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">:
+scripts/sync_docs_to_notebooklm.py </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>や</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> docs/DEVELOPMENT_KNOWLEDGE_FLOW.md: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>プロジェクト内の全</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Runbook</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>・仕様書・</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>WBS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>を</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>RAG</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ナレッジベース化し、開発者</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>QA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>応答や</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>資料生成の基盤として利用。</t>
+    </r>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>📬</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>「</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>POP3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Post Office Protocol version 3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）」の解説</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+POP3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>とは、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>**</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>「電子メールサーバーに届いた電子メールを受信端末や自動解析プログラムへ一括ダウンロード・取り込みを行うための標準ネットワークプロトコル（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>RFC 1939</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）」</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>**</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>を指します。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>💡</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>特徴と</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>IMAP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>との比較</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+POP3 (Post Office Protocol v3): </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>サーバーから未読メールをまとめてクライアント側に取得・保存して処理。ローカルでの保存・高速な一括読み込みに適しています。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+IMAP (Internet Message Access Protocol): </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>サーバー上のメール本体やフォルダ状態（未読</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>既読）を複数端末でリアルタイム同期・参照します。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>💡</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>本プロダクト（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mighty Skill-Bridge</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）での活用</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>営業メール</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>マッチング機能</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">:
+SALES_EMAIL_INGESTION_POC_RUNBOOK.md / SALES_EMAIL_EXTRACTION_PIPELINE_RUNBOOK.md:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>営業担当メールアドレス宛に届く案件情報・技術者提案メールを、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>POP3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>経由で漏れなく全件自動抽出し、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>スコアリングパイプライン（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Gemini</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）へ安全に受け渡す基本通信規格として使用されています。</t>
+    </r>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>LLM</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Emoji"/>
+        <family val="2"/>
+      </rPr>
+      <t>🧠</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>「</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>LLM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Large Language Model / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>大規模言語モデル）」の解説</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+LLM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>とは、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>**</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>「ペタバイト規模の莫大なテキストデータと深層学習（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Transformer</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>建築等）を用いて事前学習された、自然言語の理解、要約、翻訳、推論、コード生成、分類を高精度で行う人工知能（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）の基盤モデル」</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>**</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>を指します。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>💡</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>本プロダクト（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mighty Skill-Bridge</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）における主な</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>LLM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>活用</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>基盤モデルの採用（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Google Gemini </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>シリーズ）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">:
+docs/GEMINI_MODEL_VERSION_MIGRATION_RUNBOOK.md / scripts/audit_gemini_model_policy.py:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>高速・低コストな</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Gemini Flash </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>や高精度・複雑推論向けの</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Gemini Pro</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">1.5 / 2.0 / 3.1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>等）を用途に応じて最適使い分け。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>営業メール</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>マッチング</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>自然言語で送られる大量の非構造化メールから、スキル要件、稼働開始時期、契約条件、マッチングスコアを自動抽出・構造化。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>適性・モチベーション診断の自動定性サマリ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>:
+6</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>次元パラメーターを言語化し、管理者・人事担当者向けの解説テキストや面談示唆を生成。</t>
+    </r>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ハーネス</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Emoji"/>
+        <family val="2"/>
+      </rPr>
+      <t>🧪</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>「ハーネス（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Test Harness / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>テストハーネス）」の解説</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+**</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>テストハーネス（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Harness</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）とは、「プログラム、モジュール、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>モデル、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>API</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>等を独立して自動実行・検証・評価するために、テスト対象を包み込んで入力データの供給、外部依存（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>DB</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>や</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>API</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>等）のモック化、実行制御、結果の判定（アサーション）、証跡レポート出力を一括して担うテスト実行基盤・枠組み一式」</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>**</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>を指します。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>💡</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ハーネスの主な構成要素</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>テストドライバ（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Test Driver</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>テスト対象を呼び出し、引数や擬似リクエストを投入する実行機構。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>テストスタブ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>モック（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mock / Stub</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>外部依存（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Stripe</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>決済、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Google OAuth</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Supabase</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Gemini API</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>等）を擬似応答で代替し、環境に依存せずテストを完結させる仕組み。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>アサーション・検証器（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Assertions &amp; Evaluators</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>出力結果が仕様通りの型・値・ステータスかを機械的に合否判定。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>証跡・メトリクス出力</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>実行結果や網羅率をレポート（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Markdown/JSON</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>等）として自動生成。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>💡</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>本プロダクト（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mighty Skill-Bridge</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）での活用</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>レーン・プリフライト監査ハーネス</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (scripts/run_lane_preflight.py):
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>全</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>25</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>件の整合ガードと</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Pytest</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>スイート（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>120</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>超のテストファイル）を一括実行し、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>仮説（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>H1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>〜</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>H10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）に基づきリポジトリ全体の健全性を瞬時に判定・証跡化。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>・</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>API</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>契約テストハーネス</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">:
+audit_frontend_api_contract.py </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>や</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> audit_uat_api_coverage.py: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>フロントエンドとバックエンドの</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>API</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>契約や</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>UAT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>仕様をモック</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ドライバ経由で自動検証。</t>
+    </r>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>セッション</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Emoji"/>
+        <family val="2"/>
+      </rPr>
+      <t>⏱️</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>「セッション（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Session</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）」の解説</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>セッションとは、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>**</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>「システム、通信、または開発運用において、開始から終了までの一連の継続的な処理単位・対話状態」</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>**</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>を指します。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>💡</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>本プロジェクトにおける</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>つの重要文脈</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Web</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>・認証におけるセッション（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>User Auth Session</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ユーザーがログインしてからログアウト（または有効期限切れ）するまでの認証継続状態。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Firebase Auth </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>により</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> JWT / ID </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>トークンが発行・管理され、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Supabase DB </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>へのアクセス制御（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>RLS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）に安全に引き継がれます。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>開発運用におけるセッション（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Dev / Agent Session</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">:
+AGENTS.md
+ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>で定義された</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>回の開発作業単位。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>セッション規約</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>各セッションで最低</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>件の</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> WBS </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>タスク（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>data/WBS.tsv</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）を完了し、終了前に必ずプリフライト監査（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>python scripts/run_lane_preflight.py</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）を実行して作業ツリーの健全性（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>green</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）を担保します。</t>
     </r>
     <phoneticPr fontId="1"/>
   </si>
@@ -16623,7 +19838,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D61D7BD1-E21E-491C-9734-845F33AEBE13}">
-  <dimension ref="B3:E19"/>
+  <dimension ref="B3:E23"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="3.375" bestFit="1" customWidth="1"/>
@@ -16651,7 +19866,7 @@
         <v>1</v>
       </c>
       <c r="C4">
-        <f t="shared" ref="C4:C19" si="0">C3+1</f>
+        <f t="shared" ref="C4:C23" si="0">C3+1</f>
         <v>2</v>
       </c>
       <c r="D4" t="s">
@@ -16857,6 +20072,9 @@
       </c>
     </row>
     <row r="18" spans="2:5" ht="296.25" x14ac:dyDescent="0.4">
+      <c r="B18" t="s">
+        <v>1</v>
+      </c>
       <c r="C18">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -16868,13 +20086,79 @@
         <v>75</v>
       </c>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="19" spans="2:5" ht="255" x14ac:dyDescent="0.4">
+      <c r="B19" t="s">
+        <v>1</v>
+      </c>
       <c r="C19">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="D19" t="s">
         <v>72</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" ht="367.5" x14ac:dyDescent="0.4">
+      <c r="B20" t="s">
+        <v>1</v>
+      </c>
+      <c r="C20">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+      <c r="D20" t="s">
+        <v>76</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" ht="236.25" x14ac:dyDescent="0.4">
+      <c r="B21" t="s">
+        <v>1</v>
+      </c>
+      <c r="C21">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
+      <c r="D21" t="s">
+        <v>80</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" ht="333.75" x14ac:dyDescent="0.4">
+      <c r="B22" t="s">
+        <v>1</v>
+      </c>
+      <c r="C22">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="D22" t="s">
+        <v>82</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5" ht="236.25" x14ac:dyDescent="0.4">
+      <c r="B23" t="s">
+        <v>1</v>
+      </c>
+      <c r="C23">
+        <f t="shared" si="0"/>
+        <v>21</v>
+      </c>
+      <c r="D23" t="s">
+        <v>84</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -16884,6 +20168,28 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49199C90-9BB8-45C0-BAA3-6AD72AA42C11}">
+  <dimension ref="D3"/>
+  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="4" max="4" width="62.375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="4:4" x14ac:dyDescent="0.4">
+      <c r="D3" s="3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <hyperlinks>
+    <hyperlink ref="D3" r:id="rId1" xr:uid="{519012D9-D57E-4685-BBA6-CB1C8061383A}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FFF1E46-B8F1-4111-9292-CB57C462E366}">
   <dimension ref="A2:F6"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
@@ -16987,7 +20293,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3130DC33-D7DC-49CA-BAC6-4FF425438F8A}">
   <dimension ref="A2:D3"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>

</xml_diff>

<commit_message>
feat(security): add security log integrity and cost quota alerts guards, sync WBS/Sheets/Calendar
</commit_message>
<xml_diff>
--- a/mighty-link-ai-connect.xlsx
+++ b/mighty-link-ai-connect.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\mighty-link-ai-connect\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D3CFE07-1BCC-4497-99A2-4321FECC6901}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7BA0465-0B7F-4274-AE41-0C02F1337C6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{66EF4EAD-7CE3-414D-A20B-206D64169BF2}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="94">
   <si>
     <t>C:\Users\kanta\GitHub\mighty-link-ai-connect\__pycache__</t>
     <phoneticPr fontId="1"/>
@@ -19748,6 +19748,1270 @@
         <scheme val="minor"/>
       </rPr>
       <t>用語表記揺れ防止の単一正本。</t>
+    </r>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ブランチ</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>🌿</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>「ブランチ（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Branch</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）」の解説</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+**</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ブランチ（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Branch</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）とは、「</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Git </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>などのバージョン管理システムにおいて、主要な開発ライン（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">main </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ブランチ等）から履歴を分岐させ、他の作業や本番環境に影響を与えることなく新機能の実装・バグ修正・実験的コードの検証を並行して進めるための独立した作業空間」</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>**</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>を指します。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>💡</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>本プロジェクト（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mighty Skill-Bridge</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）におけるブランチ運用方針</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>本番自動デプロイ先としての</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> main </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ブランチ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">:
+main </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ブランチへのコミットやマージは、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Firebase Hosting</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>mightylink-app.com</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）へ即座に自動デプロイされるプロダクション環境直結の基幹ブランチです。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>レーン・プリフライト監査による保護</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>:
+3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>レーン体制（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Antigravity, Codex, Claude Code</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）がコードをプッシュ・マージする前に、必ずプリフライト監査（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>python scripts/run_lane_preflight.py</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）を実行して</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> 25 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>件の整合ガードと全自動テストスイートを合格（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>green</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）させることで、破損やドリフトのない健全な状態を維持します。</t>
+    </r>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>worktree</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>SES</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>🌳</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>「</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>worktree</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Git Worktree / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ワークツリー）」の解説</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Git Worktree</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>とは、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>**</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>「同一のローカル</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Git</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>リポジトリ（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>.git</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）を共有しながら、異なる複数のブランチを別の作業ディレクトリ（ワーキングツリー）として同時にチェックアウト・展開し、独立して並行作業・テスト・ビルドを実行できる</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Git</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>機能」</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>**</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>を指します。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>💡</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Worktree</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>の主な利点と特徴</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>リポジトリの再クローン不要</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ディスク容量やオブジェクト</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>DB</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>を無駄に消費せず、数秒で独立した並行作業ディレクトリを作成可能。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>作業の中断・</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>stash</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>・コンフリクト回避</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>進行中の作業を</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> git stash </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>やコミットで退避させることなく、別ディレクトリで緊急のバグ修正や別機能のテストを並行して実行可能。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>エージェント</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>サブエージェントのワークスペース分離</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>複数レーンやサブエージェント（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Antigravity, Codex</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>等）が、親ブランチの作業ツリーを汚染・競合することなく独立して安全にリサーチやコード修正を行う隔離基盤（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Workspace: 'share' </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>モード等）として活用されます。</t>
+    </r>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>💼</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>「</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>SES</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">System Engineering Service / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>システムエンジニアリングサービス）」の解説</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+**SES</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（システムエンジニアリングサービス）とは、「</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>IT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>業界における準委任契約形態のひとつであり、クライアント企業のプロジェクトやシステム開発に対して、エンジニアの技術力・労働力を継続的に提供・支援するサービス形態」</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>**</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>を指します。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>💡</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>本プロダクト（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mighty Skill-Bridge</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）との深い関わり</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>業界特有の課題（営業メールの山）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>:
+SES</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>業界では、毎日数千通規模で「案件募集メール」やパートナー企業からの「エンジニア提案メール（スキルシート）」が送受信され、営業担当者が目視で突き合わせ作業を行っています。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>営業メール</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>マッチングによる</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>DX:
+docs/SALES_EMAIL_AI_MATCHING_REQUIREMENTS.md / SALES_EMAIL_INGESTION_POC_RUNBOOK.md:
+POP3/IMAP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>経由で受信したメールを</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Gemini LLM </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>が全件自動解析し、必要スキル・稼働時期・単価条件を即座に判定・スコアリング。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+North Star KPI </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>である「営業マッチング成約時間の削減率」を劇的に改善する中核ターゲット領域となっています。</t>
     </r>
     <phoneticPr fontId="1"/>
   </si>
@@ -20346,7 +21610,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D61D7BD1-E21E-491C-9734-845F33AEBE13}">
-  <dimension ref="B3:E24"/>
+  <dimension ref="B3:E27"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="3.375" bestFit="1" customWidth="1"/>
@@ -20374,7 +21638,7 @@
         <v>1</v>
       </c>
       <c r="C4">
-        <f t="shared" ref="C4:C24" si="0">C3+1</f>
+        <f t="shared" ref="C4:C27" si="0">C3+1</f>
         <v>2</v>
       </c>
       <c r="D4" t="s">
@@ -20684,6 +21948,51 @@
         <v>87</v>
       </c>
     </row>
+    <row r="25" spans="2:5" ht="240" x14ac:dyDescent="0.4">
+      <c r="B25" t="s">
+        <v>1</v>
+      </c>
+      <c r="C25">
+        <f t="shared" si="0"/>
+        <v>23</v>
+      </c>
+      <c r="D25" t="s">
+        <v>88</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="26" spans="2:5" ht="258.75" x14ac:dyDescent="0.4">
+      <c r="B26" t="s">
+        <v>1</v>
+      </c>
+      <c r="C26">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+      <c r="D26" t="s">
+        <v>90</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="27" spans="2:5" ht="236.25" x14ac:dyDescent="0.4">
+      <c r="B27" t="s">
+        <v>1</v>
+      </c>
+      <c r="C27">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+      <c r="D27" t="s">
+        <v>91</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix(hooks): full official Antigravity Stop lifecycle contract, PII redaction, deduplication, and UI test stability
</commit_message>
<xml_diff>
--- a/mighty-link-ai-connect.xlsx
+++ b/mighty-link-ai-connect.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\mighty-link-ai-connect\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18D77A0B-E2F8-4D45-B63A-949C29728EAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDD09742-60EE-42AB-979E-B490B2408EA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{66EF4EAD-7CE3-414D-A20B-206D64169BF2}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="103">
   <si>
     <t>C:\Users\kanta\GitHub\mighty-link-ai-connect\__pycache__</t>
     <phoneticPr fontId="1"/>
@@ -22155,6 +22155,10 @@
       </rPr>
       <t>）および価値提案・機能説明セクションの直後に反復配置。</t>
     </r>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>1.2 Learn with ChatGPT</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -23173,7 +23177,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49199C90-9BB8-45C0-BAA3-6AD72AA42C11}">
-  <dimension ref="B2:G3"/>
+  <dimension ref="B2:G4"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="2.5" bestFit="1" customWidth="1"/>
@@ -23207,6 +23211,11 @@
       </c>
       <c r="G3" t="s">
         <v>94</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="G4" t="s">
+        <v>102</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(ci): register audit_sessions.py in exempt guards in run_lane_preflight.py
</commit_message>
<xml_diff>
--- a/mighty-link-ai-connect.xlsx
+++ b/mighty-link-ai-connect.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\mighty-link-ai-connect\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDD09742-60EE-42AB-979E-B490B2408EA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33C1A4FE-1E76-4140-B405-928286DFA369}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{66EF4EAD-7CE3-414D-A20B-206D64169BF2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{66EF4EAD-7CE3-414D-A20B-206D64169BF2}"/>
   </bookViews>
   <sheets>
     <sheet name="ソースコードレビュー" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="105">
   <si>
     <t>C:\Users\kanta\GitHub\mighty-link-ai-connect\__pycache__</t>
     <phoneticPr fontId="1"/>
@@ -22159,6 +22159,791 @@
   </si>
   <si>
     <t>1.2 Learn with ChatGPT</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>SRE</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Emoji"/>
+        <family val="2"/>
+      </rPr>
+      <t>🛠️</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>「</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>SRE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Site Reliability Engineering / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>サイト信頼性エンジニアリング）」の解説</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+**SRE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（サイト信頼性エンジニアリング）とは、「</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Google </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>が提唱したシステム運用の規律・手法であり、ソフトウェア工学（ソフトウェア開発のアプローチ）を用いてインフラ・サービスの可用性、耐障害性、パフォーマンス、スケーラビリティを継続的に向上させる実践体系」</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>**</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>を指します。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>💡</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>SRE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>の重要コア概念</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+SLI / SLO / SLA:
+SLI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（指標）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>可用性やレスポンス速度の実測値。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+SLO</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（目標）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>チームが目指す信頼性目標（例</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>可用性</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> 99.9%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+SLA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（合意）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>顧客・ユーザーに対して保証する契約基準。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>トイル（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Toil</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）の撲滅</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>手作業で反復される定常業務を、自動化スクリプトや</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>CI/CD</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>パイプラインによって最小化。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>障害ポストモーテム（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Blameless Postmortem</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>障害原因を個人の過失に求めず、システムの構造的欠陥や手順不備を分析して再発防止を図る文化。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>💡</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>本プロジェクト（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mighty Skill-Bridge</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）における主な</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>SRE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>実践</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+DevOps / SRE </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>運用仕様書</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">:
+docs/DEVOPS_SRE_OPERATION_SPEC.md
+ / 
+docs/SLA_KPI_DEFINITION_AND_MEASUREMENT.md
+: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>可用性目標とレスポンス監視の規定。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>全</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>46</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>本の運用</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Runbook</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>カタログ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">:
+docs/OPERATIONS_RUNBOOK_CATALOG.md
+: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>バックアップ、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>DB</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>マイグレーション、障害復旧手順を体系化。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>自動品質・整合性ガード（レーン・プリフライト監査）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>リポジトリのドリフトを即座に機械検知する自動化</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>CI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>装置。</t>
+    </r>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -22756,7 +23541,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D61D7BD1-E21E-491C-9734-845F33AEBE13}">
-  <dimension ref="B3:E29"/>
+  <dimension ref="B3:E30"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="3.375" bestFit="1" customWidth="1"/>
@@ -22784,7 +23569,7 @@
         <v>1</v>
       </c>
       <c r="C4">
-        <f t="shared" ref="C4:C29" si="0">C3+1</f>
+        <f t="shared" ref="C4:C30" si="0">C3+1</f>
         <v>2</v>
       </c>
       <c r="D4" t="s">
@@ -23169,6 +23954,21 @@
         <v>101</v>
       </c>
     </row>
+    <row r="30" spans="2:5" ht="409.5" x14ac:dyDescent="0.4">
+      <c r="B30" t="s">
+        <v>1</v>
+      </c>
+      <c r="C30">
+        <f t="shared" si="0"/>
+        <v>28</v>
+      </c>
+      <c r="D30" t="s">
+        <v>103</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>104</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
audit stalled work and harden launch evidence
</commit_message>
<xml_diff>
--- a/mighty-link-ai-connect.xlsx
+++ b/mighty-link-ai-connect.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\mighty-link-ai-connect\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81706E12-1C70-432B-80EA-4FA95A015B7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3384C427-AD29-4F0C-9FE0-D7E5AD76B984}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{66EF4EAD-7CE3-414D-A20B-206D64169BF2}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="113">
   <si>
     <t>C:\Users\kanta\GitHub\mighty-link-ai-connect\__pycache__</t>
     <phoneticPr fontId="1"/>
@@ -22956,6 +22956,26 @@
   </si>
   <si>
     <t>1.3 Check-in</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>2.1 What is AI?</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=QJ-oM6DcMz4</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=ejHBZzoZxRs</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>2.2 What LLMs can do</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=QfyU7N4aVTg</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -23995,7 +24015,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49199C90-9BB8-45C0-BAA3-6AD72AA42C11}">
-  <dimension ref="B2:H5"/>
+  <dimension ref="B2:H7"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="2.5" bestFit="1" customWidth="1"/>
@@ -24042,10 +24062,29 @@
       <c r="G4" t="s">
         <v>102</v>
       </c>
+      <c r="H4" s="3" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.4">
       <c r="G5" t="s">
         <v>107</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="G6" t="s">
+        <v>108</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="G7" t="s">
+        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -24055,6 +24094,9 @@
     <hyperlink ref="E3" r:id="rId2" xr:uid="{105F50FE-3BAA-4EAE-867D-A196B32BB119}"/>
     <hyperlink ref="H3" r:id="rId3" xr:uid="{F9F88046-A983-43FE-A30C-07771C0C5A43}"/>
     <hyperlink ref="F3" r:id="rId4" xr:uid="{10580E7B-8AA3-47D8-942A-F28AB2887FD5}"/>
+    <hyperlink ref="H4" r:id="rId5" xr:uid="{03BB2B03-8C36-4017-A518-CE3BC314953D}"/>
+    <hyperlink ref="H5" r:id="rId6" xr:uid="{5F2D1BB3-51D2-4792-8A97-B48004C15BAA}"/>
+    <hyperlink ref="H6" r:id="rId7" xr:uid="{1E91F52D-EDCF-444F-A15C-D01E5DA67DFC}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(matching): add mailto launcher, P0/P1/P2 roadmap improvements, and safe IMAP sync
</commit_message>
<xml_diff>
--- a/mighty-link-ai-connect.xlsx
+++ b/mighty-link-ai-connect.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\mighty-link-ai-connect\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3384C427-AD29-4F0C-9FE0-D7E5AD76B984}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D961B93-EE3D-4870-AAD7-39E9CF2B007E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{66EF4EAD-7CE3-414D-A20B-206D64169BF2}"/>
   </bookViews>
@@ -18,6 +18,7 @@
     <sheet name="OpenAIAcademy" sheetId="5" r:id="rId3"/>
     <sheet name="YouTube" sheetId="3" r:id="rId4"/>
     <sheet name="ブログ" sheetId="4" r:id="rId5"/>
+    <sheet name="令和の虎" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="141">
   <si>
     <t>C:\Users\kanta\GitHub\mighty-link-ai-connect\__pycache__</t>
     <phoneticPr fontId="1"/>
@@ -22978,12 +22979,155 @@
     <t>https://www.youtube.com/watch?v=QfyU7N4aVTg</t>
     <phoneticPr fontId="1"/>
   </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=ZFVlTcRwNVU</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=KWURBiF0kAs</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>FAL</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>HEDRA</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>2.3 How models are trained</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>2.4 Know when to use trusted sources</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=5wVvLi-H8PE</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=VqCeYy7yg28</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>2.5 Why AI needs human review</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Runway</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ElevenLabs</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Seedance</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Veo</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=rSjdyQv1Wfc</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <r>
+      <t>【マネ虎だった人々#001マネーの虎　現在の姿［南原社長①］】記念すべき初回ゲストはあの</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>‪</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>@nambara</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>‬</t>
+    </r>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=ib7mIx5p7Wo</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>2.6 Check-in</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=vLTQ_iJuhho</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>3.1 Why clear instructions matter</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=2rzqAjG6Ih8</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>3.2 Task, Concept, and Expectation</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Adobe Firefly Services</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Luma Dream Machine</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>HeyGen</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Topaz Video AI</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Synthesia</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Tavus</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Shotstack</t>
+    <phoneticPr fontId="1"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -23032,6 +23176,12 @@
       <family val="2"/>
       <charset val="128"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -24015,7 +24165,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49199C90-9BB8-45C0-BAA3-6AD72AA42C11}">
-  <dimension ref="B2:H7"/>
+  <dimension ref="B2:J19"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="2.5" bestFit="1" customWidth="1"/>
@@ -24023,11 +24173,12 @@
     <col min="4" max="4" width="62.375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="49.625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="78.75" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="30" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="36.875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="50.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:10" x14ac:dyDescent="0.4">
       <c r="E2" t="s">
         <v>96</v>
       </c>
@@ -24035,7 +24186,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:10" x14ac:dyDescent="0.4">
       <c r="B3">
         <v>1</v>
       </c>
@@ -24058,7 +24209,10 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:10" x14ac:dyDescent="0.4">
+      <c r="F4" t="s">
+        <v>1</v>
+      </c>
       <c r="G4" t="s">
         <v>102</v>
       </c>
@@ -24066,7 +24220,10 @@
         <v>109</v>
       </c>
     </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.4">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.4">
+      <c r="F5" t="s">
+        <v>1</v>
+      </c>
       <c r="G5" t="s">
         <v>107</v>
       </c>
@@ -24074,7 +24231,10 @@
         <v>110</v>
       </c>
     </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:10" x14ac:dyDescent="0.4">
+      <c r="F6" t="s">
+        <v>1</v>
+      </c>
       <c r="G6" t="s">
         <v>108</v>
       </c>
@@ -24082,9 +24242,156 @@
         <v>112</v>
       </c>
     </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.4">
+    <row r="7" spans="2:10" x14ac:dyDescent="0.4">
+      <c r="F7" t="s">
+        <v>1</v>
+      </c>
       <c r="G7" t="s">
         <v>111</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="I7" t="s">
+        <v>116</v>
+      </c>
+      <c r="J7" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="2:10" x14ac:dyDescent="0.4">
+      <c r="F8" t="s">
+        <v>1</v>
+      </c>
+      <c r="G8" t="s">
+        <v>111</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="I8" t="s">
+        <v>115</v>
+      </c>
+      <c r="J8" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="2:10" x14ac:dyDescent="0.4">
+      <c r="F9" t="s">
+        <v>1</v>
+      </c>
+      <c r="G9" t="s">
+        <v>117</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="I9" t="s">
+        <v>122</v>
+      </c>
+      <c r="J9" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="2:10" x14ac:dyDescent="0.4">
+      <c r="F10" t="s">
+        <v>1</v>
+      </c>
+      <c r="G10" t="s">
+        <v>118</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="I10" t="s">
+        <v>123</v>
+      </c>
+      <c r="J10" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="2:10" x14ac:dyDescent="0.4">
+      <c r="F11" t="s">
+        <v>1</v>
+      </c>
+      <c r="G11" t="s">
+        <v>121</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="I11" t="s">
+        <v>124</v>
+      </c>
+      <c r="J11" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="2:10" x14ac:dyDescent="0.4">
+      <c r="F12" t="s">
+        <v>1</v>
+      </c>
+      <c r="G12" t="s">
+        <v>129</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="I12" t="s">
+        <v>125</v>
+      </c>
+      <c r="J12" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="2:10" x14ac:dyDescent="0.4">
+      <c r="F13" t="s">
+        <v>1</v>
+      </c>
+      <c r="G13" t="s">
+        <v>131</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="I13" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="14" spans="2:10" x14ac:dyDescent="0.4">
+      <c r="G14" t="s">
+        <v>133</v>
+      </c>
+      <c r="I14" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="15" spans="2:10" x14ac:dyDescent="0.4">
+      <c r="I15" t="s">
+        <v>136</v>
+      </c>
+      <c r="J15" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="2:10" x14ac:dyDescent="0.4">
+      <c r="I16" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="17" spans="9:9" x14ac:dyDescent="0.4">
+      <c r="I17" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="18" spans="9:9" x14ac:dyDescent="0.4">
+      <c r="I18" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="19" spans="9:9" x14ac:dyDescent="0.4">
+      <c r="I19" t="s">
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -24097,6 +24404,13 @@
     <hyperlink ref="H4" r:id="rId5" xr:uid="{03BB2B03-8C36-4017-A518-CE3BC314953D}"/>
     <hyperlink ref="H5" r:id="rId6" xr:uid="{5F2D1BB3-51D2-4792-8A97-B48004C15BAA}"/>
     <hyperlink ref="H6" r:id="rId7" xr:uid="{1E91F52D-EDCF-444F-A15C-D01E5DA67DFC}"/>
+    <hyperlink ref="H7" r:id="rId8" xr:uid="{0D564E43-38C4-48F4-AAAB-4525354FC72F}"/>
+    <hyperlink ref="H8" r:id="rId9" xr:uid="{C0D26131-7E05-42BC-82C1-BF5A3C8CA0AA}"/>
+    <hyperlink ref="H9" r:id="rId10" xr:uid="{064DA19D-7439-463F-82FE-C95706338D47}"/>
+    <hyperlink ref="H10" r:id="rId11" xr:uid="{14228D45-42B2-48B7-925F-FA241A01441B}"/>
+    <hyperlink ref="H11" r:id="rId12" xr:uid="{367E638D-234E-4EDB-AEF7-C988D3EC6D19}"/>
+    <hyperlink ref="H12" r:id="rId13" xr:uid="{1F218158-2EA3-4B0C-BF90-D126C575D2B6}"/>
+    <hyperlink ref="H13" r:id="rId14" xr:uid="{4ED2049A-D59E-4607-9BBE-3F4210108A82}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -24221,7 +24535,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="93.75" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" s="2">
         <v>46248</v>
       </c>
@@ -24242,4 +24556,34 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C864D64-BD4E-47C2-98A7-786282D674DD}">
+  <dimension ref="B3:D3"/>
+  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="2" max="2" width="2.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="48.25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="98.375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.4">
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <hyperlinks>
+    <hyperlink ref="C3" r:id="rId1" xr:uid="{2979877C-AB48-4013-966B-133B0CF0552C}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: complete phase 7 autopilot bridge, external platform hub, and 8/24 go/no-go audit (T994, T995)
</commit_message>
<xml_diff>
--- a/mighty-link-ai-connect.xlsx
+++ b/mighty-link-ai-connect.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\mighty-link-ai-connect\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D961B93-EE3D-4870-AAD7-39E9CF2B007E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54D25E2F-FB33-4DF8-B3A4-C308A510F000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{66EF4EAD-7CE3-414D-A20B-206D64169BF2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{66EF4EAD-7CE3-414D-A20B-206D64169BF2}"/>
   </bookViews>
   <sheets>
     <sheet name="ソースコードレビュー" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="142">
   <si>
     <t>C:\Users\kanta\GitHub\mighty-link-ai-connect\__pycache__</t>
     <phoneticPr fontId="1"/>
@@ -23120,6 +23120,597 @@
   </si>
   <si>
     <t>Shotstack</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Emoji"/>
+        <family val="2"/>
+      </rPr>
+      <t>🛠️</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>「</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>SRE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Site Reliability Engineering</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）」の解説</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+**SRE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（サイト信頼性エンジニアリング）とは、「</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Google </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>が提唱したシステム運用の規律・手法であり、ソフトウェア工学のアプローチを用いて、インフラ・</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Web</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>サービスの可用性、耐障害性、パフォーマンス、スケーラビリティを継続的に向上・維持させる実践体系」</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>**</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>を指します。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>💡</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>SRE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>の重要コア要素</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>定量的サービスレベル管理</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>:
+SLI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Service Level Indicator</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>実際の稼働率やレスポンス速度の測定指標。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+SLO</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Service Level Objective</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>チームが目指す信頼性目標（例</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>可用性</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> 99.9%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+SLA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Service Level Agreement</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>顧客へ保証する契約合意。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>トイル（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Toil</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）の撲滅</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>繰り返される手作業の運用業務を、自動化スクリプトや</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>CI/CD</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>パイプラインにより最小化。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>エラーバジェット（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Error Budget</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>許容される不稼働時間の枠を定義し、新機能リリース速度と安定性のバランスを最適化。</t>
+    </r>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -24151,10 +24742,16 @@
         <v>104</v>
       </c>
     </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="31" spans="2:5" ht="258.75" x14ac:dyDescent="0.4">
       <c r="C31">
         <f t="shared" si="0"/>
         <v>29</v>
+      </c>
+      <c r="D31" t="s">
+        <v>103</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>141</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(tool-lanes): update tool lane names to Codex and Claude Code and align docs/WBS
</commit_message>
<xml_diff>
--- a/mighty-link-ai-connect.xlsx
+++ b/mighty-link-ai-connect.xlsx
@@ -1,24 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\mighty-link-ai-connect\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D961B93-EE3D-4870-AAD7-39E9CF2B007E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9C916C7-DD21-4C33-8943-61B83AF8B9E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{66EF4EAD-7CE3-414D-A20B-206D64169BF2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{66EF4EAD-7CE3-414D-A20B-206D64169BF2}"/>
   </bookViews>
   <sheets>
     <sheet name="ソースコードレビュー" sheetId="1" r:id="rId1"/>
     <sheet name="用語集" sheetId="2" r:id="rId2"/>
     <sheet name="OpenAIAcademy" sheetId="5" r:id="rId3"/>
-    <sheet name="YouTube" sheetId="3" r:id="rId4"/>
-    <sheet name="ブログ" sheetId="4" r:id="rId5"/>
-    <sheet name="令和の虎" sheetId="6" r:id="rId6"/>
+    <sheet name="Antigravity" sheetId="7" r:id="rId4"/>
+    <sheet name="ClaudeAcademy" sheetId="8" r:id="rId5"/>
+    <sheet name="YouTube" sheetId="3" r:id="rId6"/>
+    <sheet name="ブログ" sheetId="4" r:id="rId7"/>
+    <sheet name="令和の虎" sheetId="6" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="193">
   <si>
     <t>C:\Users\kanta\GitHub\mighty-link-ai-connect\__pycache__</t>
     <phoneticPr fontId="1"/>
@@ -16035,10 +16037,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>https://academy.openai.com/learn/ai-foundations-juzjs/lessons</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -21014,14 +21012,6 @@
       </rPr>
       <t>である「営業マッチング成約時間の削減率」を劇的に改善する中核ターゲット領域となっています。</t>
     </r>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>1.1 Welcome to AI Foundations</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>https://www.youtube.com/watch?v=yAbco3K_TLQ</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
@@ -22159,10 +22149,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>1.2 Learn with ChatGPT</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>SRE</t>
     <phoneticPr fontId="1"/>
   </si>
@@ -22945,90 +22931,6 @@
       </rPr>
       <t>装置。</t>
     </r>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>https://www.youtube.com/watch?v=yGCLS7EW91A</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>https://notebook.google.com/notebook/442dbe89-a27d-4b73-a330-4baa0652370c</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>1.3 Check-in</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>2.1 What is AI?</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>https://www.youtube.com/watch?v=QJ-oM6DcMz4</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>https://www.youtube.com/watch?v=ejHBZzoZxRs</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>2.2 What LLMs can do</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>https://www.youtube.com/watch?v=QfyU7N4aVTg</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>https://www.youtube.com/watch?v=ZFVlTcRwNVU</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>https://www.youtube.com/watch?v=KWURBiF0kAs</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>FAL</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>HEDRA</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>2.3 How models are trained</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>2.4 Know when to use trusted sources</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>https://www.youtube.com/watch?v=5wVvLi-H8PE</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>https://www.youtube.com/watch?v=VqCeYy7yg28</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>2.5 Why AI needs human review</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>Runway</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>ElevenLabs</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>Seedance</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>Veo</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
@@ -23071,55 +22973,2592 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>https://www.youtube.com/watch?v=ib7mIx5p7Wo</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Emoji"/>
+        <family val="2"/>
+      </rPr>
+      <t>🛠️</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>「</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>SRE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Site Reliability Engineering</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）」の解説</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+**SRE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（サイト信頼性エンジニアリング）とは、「</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Google </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>が提唱したシステム運用の規律・手法であり、ソフトウェア工学のアプローチを用いて、インフラ・</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Web</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>サービスの可用性、耐障害性、パフォーマンス、スケーラビリティを継続的に向上・維持させる実践体系」</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>**</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>を指します。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>💡</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>SRE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>の重要コア要素</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>定量的サービスレベル管理</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>:
+SLI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Service Level Indicator</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>実際の稼働率やレスポンス速度の測定指標。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+SLO</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Service Level Objective</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>チームが目指す信頼性目標（例</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>可用性</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> 99.9%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+SLA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Service Level Agreement</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>顧客へ保証する契約合意。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>トイル（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Toil</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）の撲滅</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>繰り返される手作業の運用業務を、自動化スクリプトや</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>CI/CD</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>パイプラインにより最小化。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>エラーバジェット（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Error Budget</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>許容される不稼働時間の枠を定義し、新機能リリース速度と安定性のバランスを最適化。</t>
+    </r>
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>2.6 Check-in</t>
+    <t>アドホック</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>https://www.youtube.com/watch?v=vLTQ_iJuhho</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>🎯</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>「アドホック（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Ad-hoc / Ad hoc</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）」の解説</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>アドホックとは、ラテン語で「特定の目的のための」「その場限りの（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>for this purpose only</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）」を意味し、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>IT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>・ソフトウェア開発分野では</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>**</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>「事前の計画や定型化された手順によらず、その場限りの必要性に応じて臨機応変・単発で作成・実行される処理や対応」</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>**</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>を指します。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>💡</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>代表的な文脈・使われ方</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>アドホッククエリ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>アドホック集計</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (Ad-hoc Query):
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>定常的なバッチ処理やダッシュボード画面ではなく、特定のデータ調査・トラブルシューティング・意思決定のためにその都度単発で実行される</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>SQL</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>クエリやスクリプト。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>アドホックテスト</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (Ad-hoc Testing):
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>定義済みのテスト仕様書（テストケース）に沿わず、エンジニアやテスターが即興的・探索的に</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>UI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>や機能を触って予期せぬバグを見つけ出すテスト手法。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>アドホック対応（暫定対応</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> / Workaround</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>障害発生時や急ぎの仕様変更時に、恒久的なシステム改修の前に一時的に行われる手動操作や暫定パッチ。</t>
+    </r>
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>3.1 Why clear instructions matter</t>
+    <t>https://www.youtube.com/watch?v=e323zNN2lgI</t>
+  </si>
+  <si>
+    <t>3.3 Review the output</t>
+  </si>
+  <si>
+    <t>〇</t>
+  </si>
+  <si>
+    <t>LUFS</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>https://www.youtube.com/watch?v=2rzqAjG6Ih8</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>3.2 Task, Concept, and Expectation</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>🔊</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>「</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>LUFS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Loudness Units relative to Full Scale</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）」の解説</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+LUFS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（ラウドネス・ユニット・フルスケール）とは、音響・放送・動画配信・音楽制作において</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>**</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>「人間の耳の聴覚特性（周波数による音の聞こえやすさの偏り）を考慮し、実際に人間が感じる音の大きさ（体感音量）を測定・数値化した国際標準単位（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>ITU-R BS.1770 / EBU R128</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）」</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>**</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>です。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="MS UI Gothic"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>※</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>放送規格では</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> LKFS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Loudness, K-weighted, relative to Full Scale</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）とも呼ばれ、実質的に同一の指標です。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>💡</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>なぜ従来の「</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>dB</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（デシベル）」ではなく「</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>LUFS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>」を使うのか？</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>従来のピークメーター（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>dBFS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>音声信号の「電気的な最大振幅」を測るため、瞬間的な一発の破裂音でも高い数値が出ますが、人間が聴いたときの「全体的なうるささ・音圧」とは一致しませんでした。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ラウドネスメーター（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>LUFS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>人間の耳が感度の高い中高音域（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>〜</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>4kHz</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>付近）を強調するフィルタ（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>K</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>特性フィルタ）を通し、時間的な平均音圧を測定するため、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>**</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>「実際に聴いたときの音量感」</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>**</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>を正確に統一できます。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>💡</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>代表的な配信プラットフォームのラウドネス基準値</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>各プラットフォームでは、動画や楽曲ごとに急に音が大きくなったり小さくなったりするのを防ぐため、自動ノーマライズ（音量自動調整）を行っています。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>プラットフォーム</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>媒体</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">	</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>基準ラウドネス値</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (Target LUFS)	</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>備考</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+YouTube	-14 LUFS	</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>超過した音声は自動でボリュームが下げられる</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Spotify	-14 LUFS	</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>標準ノーマライズ設定</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Apple Music	-16 LUFS	Sound Check </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>機能の基準</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ポッドキャスト</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>音声配信</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">	-16 LUFS (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ステレオ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>) / -19 LUFS (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>モノラル</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">)	</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>トーク主体の標準推奨値</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>テレビ放送（日本・</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>ARIB TR-B32</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">	-24 LUFS	CM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>と番組本編の音量差を規制する基準</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>💡</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> 3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>つの測定モード</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Integrated LUFS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（統合ラウドネス）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>音声・動画全体の通算平均音量（マスタリングの最終ターゲット）。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Short-term LUFS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（短期ラウドネス）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>直近</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>秒間の音量推移。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Momentary LUFS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（瞬間ラウドネス）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>直近</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>400</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ミリ秒の瞬間的な音量感。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>💡</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>本プロジェクト（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mighty Skill-Bridge</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）や</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>AI/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>メディアにおける関連性</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>動画デモ・プロモーション動画・ナレーション生成</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>プロダクト紹介動画や</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> NotebookLM </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>等による音声解説（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Audio Overview</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）を配信する際、リスナーにとって快適で聴き取りやすい音響バランス（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">-14 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>〜</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> -16 LUFS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）を保つための音響マスタリング基準として扱われます。</t>
+    </r>
     <phoneticPr fontId="1"/>
   </si>
   <si>
     <t>Adobe Firefly Services</t>
+  </si>
+  <si>
+    <t>https://antigravity.google/docs/home/</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Welcome to Google Antigravity</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
     <t>Luma Dream Machine</t>
+  </si>
+  <si>
+    <t>OpenAI Academy 学習管理</t>
+  </si>
+  <si>
+    <t>講座リンク、レッスン動画、関連AIツールを用途別に整理</t>
+  </si>
+  <si>
+    <t>講座概要</t>
+  </si>
+  <si>
+    <t>No.</t>
+  </si>
+  <si>
+    <t>講座名</t>
+  </si>
+  <si>
+    <t>Academy URL</t>
+  </si>
+  <si>
+    <t>YouTube投稿 URL</t>
+  </si>
+  <si>
+    <t>NotebookLM URL</t>
+  </si>
+  <si>
+    <t>1.1 Welcome to AI Foundations</t>
+  </si>
+  <si>
+    <t>https://academy.openai.com/learn/ai-foundations-juzjs/lessons</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=yAbco3K_TLQ</t>
+  </si>
+  <si>
+    <t>https://notebook.google.com/notebook/442dbe89-a27d-4b73-a330-4baa0652370c</t>
+  </si>
+  <si>
+    <t>レッスン動画</t>
+  </si>
+  <si>
+    <t>レッスン名</t>
+  </si>
+  <si>
+    <t>YouTube URL</t>
+  </si>
+  <si>
+    <t>NotebookLM</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=yGCLS7EW91A</t>
+  </si>
+  <si>
+    <t>1.2 Learn with ChatGPT</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=QJ-oM6DcMz4</t>
+  </si>
+  <si>
+    <t>1.3 Check-in</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=ejHBZzoZxRs</t>
+  </si>
+  <si>
+    <t>2.1 What is AI?</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=QfyU7N4aVTg</t>
+  </si>
+  <si>
+    <t>2.2 What LLMs can do</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=ZFVlTcRwNVU</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=KWURBiF0kAs</t>
+  </si>
+  <si>
+    <t>2.3 How models are trained</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=5wVvLi-H8PE</t>
+  </si>
+  <si>
+    <t>2.4 Know when to use trusted sources</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=VqCeYy7yg28</t>
+  </si>
+  <si>
+    <t>2.5 Why AI needs human review</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=ib7mIx5p7Wo</t>
+  </si>
+  <si>
+    <t>2.6 Check-in</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=vLTQ_iJuhho</t>
+  </si>
+  <si>
+    <t>3.1 Why clear instructions matter</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=2rzqAjG6Ih8</t>
+  </si>
+  <si>
+    <t>3.2 Task, Concept, and Expectation</t>
+  </si>
+  <si>
+    <t>関連AIツール</t>
+  </si>
+  <si>
+    <t>ツール名</t>
+  </si>
+  <si>
+    <t>確認済み</t>
+  </si>
+  <si>
+    <t>HEDRA</t>
+  </si>
+  <si>
+    <t>FAL</t>
+  </si>
+  <si>
+    <t>Runway</t>
+  </si>
+  <si>
+    <t>ElevenLabs</t>
+  </si>
+  <si>
+    <t>Seedance</t>
+  </si>
+  <si>
+    <t>Veo</t>
+  </si>
+  <si>
+    <t>HeyGen</t>
+  </si>
+  <si>
+    <t>Topaz Video AI</t>
+  </si>
+  <si>
+    <t>Synthesia</t>
+  </si>
+  <si>
+    <t>Tavus</t>
+  </si>
+  <si>
+    <t>Shotstack</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=pKfb0oox3_8</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>HeyGen</t>
+    <t>https://notebook.google.com/notebook/bf99897b-fe4d-474e-a25b-22f3bd1da24f</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>Topaz Video AI</t>
+    <t>Antigravity 2.0</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>Synthesia</t>
+    <t>https://antigravity.google/docs/overview/</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>Tavus</t>
+    <t>Google Flow</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>Shotstack</t>
+    <t>サブスク</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>あり</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>なし</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Welcome to Claude Academy</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://academy.claude.com/</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=4rxcDyniuNw</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://academy.claude.com/ja/courses/claude-code-101</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Claude Code 101</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://notebook.google.com/notebook/4ab6b6f9-5fe9-4073-9a53-85321260807b</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=Pe-2A1Rq6Hc</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Getting Started with Antigravity 2.0</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://antigravity.google/docs/getting-started/</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://academy.claude.com/ja/courses/claude-code-101/what-is-claude-code</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Claude Codeとは？</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=BjOtCEYRzmc</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://academy.claude.com/ja/courses/claude-code-101/how-claude-code-works</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Claude Codeの仕組み</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>AI大学</t>
+    <rPh sb="2" eb="4">
+      <t>ダイガク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>〇</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://academy.claude.com/ja/courses/claude-code-101/installing-claude-code</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Claude Codeのインストール</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=wqjrEI6GcYE</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -23127,7 +25566,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -23183,13 +25622,59 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="MS UI Gothic"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="游ゴシック"/>
+      <family val="2"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color rgb="FF666666"/>
+      <name val="游ゴシック"/>
+      <family val="2"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="游ゴシック"/>
+      <family val="2"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF5B9BD5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -23209,7 +25694,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -23222,12 +25707,113 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="ハイパーリンク" xfId="1" builtinId="8"/>
     <cellStyle name="標準" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="20">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF375623"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFE2F0D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF375623"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFE2F0D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <alignment vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <alignment horizontal="center" vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <alignment horizontal="center" vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -23238,6 +25824,45 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4F3C1F5F-7B96-42FA-AE6C-FCDEA3288098}" name="OpenAIAcademyOverview" displayName="OpenAIAcademyOverview" ref="A4:E5" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
+  <autoFilter ref="A4:E5" xr:uid="{4F3C1F5F-7B96-42FA-AE6C-FCDEA3288098}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{EB1159DB-4DFE-4D42-AF05-DA1405FC8D97}" name="No." dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{66ABA36C-6198-4013-964A-D8514779FE6E}" name="講座名" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{7E592AD6-6191-4740-AA50-AB5A546AA082}" name="Academy URL" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{5EB4DC8E-DCEA-40A7-94FE-1257F53672C2}" name="YouTube投稿 URL" dataDxfId="14"/>
+    <tableColumn id="5" xr3:uid="{773821AD-4E74-4982-A268-36D7B5B061EE}" name="NotebookLM URL" dataDxfId="13"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5E690145-DFD4-4608-B746-B8BC87AAEC0B}" name="OpenAIAcademyLessons" displayName="OpenAIAcademyLessons" ref="A8:D21" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
+  <autoFilter ref="A8:D21" xr:uid="{5E690145-DFD4-4608-B746-B8BC87AAEC0B}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{6AA3F78C-DA07-46F2-860F-03A202FEA960}" name="No." dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{72690B91-8717-4401-A620-375C4A4CF651}" name="レッスン名" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{DF1DC285-847F-4B9C-91F1-48BD62111A11}" name="YouTube URL" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{669A9F1A-DAF8-48C6-898B-396F9166EF9E}" name="NotebookLM" dataDxfId="7"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{1705A361-A975-42B5-ABF7-C5EB161CB3D0}" name="OpenAIAcademyTools" displayName="OpenAIAcademyTools" ref="A24:C38" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
+  <autoFilter ref="A24:C38" xr:uid="{1705A361-A975-42B5-ABF7-C5EB161CB3D0}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{0BD1BA68-9FC1-4B0F-9467-16FCF66D49D3}" name="ツール名" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{3D1F0461-BB36-47B2-A727-7B1226345334}" name="確認済み" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{5BAF893C-F8A2-442E-87F6-9737E05D3C0F}" name="サブスク" dataDxfId="2"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -23723,7 +26348,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D61D7BD1-E21E-491C-9734-845F33AEBE13}">
-  <dimension ref="B3:E31"/>
+  <dimension ref="B3:E33"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="3.375" bestFit="1" customWidth="1"/>
@@ -23751,7 +26376,7 @@
         <v>1</v>
       </c>
       <c r="C4">
-        <f t="shared" ref="C4:C31" si="0">C3+1</f>
+        <f t="shared" ref="C4:C33" si="0">C3+1</f>
         <v>2</v>
       </c>
       <c r="D4" t="s">
@@ -23983,7 +26608,7 @@
         <v>72</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="20" spans="2:5" ht="367.5" x14ac:dyDescent="0.4">
@@ -23998,7 +26623,7 @@
         <v>76</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="21" spans="2:5" ht="236.25" x14ac:dyDescent="0.4">
@@ -24010,10 +26635,10 @@
         <v>19</v>
       </c>
       <c r="D21" t="s">
+        <v>79</v>
+      </c>
+      <c r="E21" s="1" t="s">
         <v>80</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="22" spans="2:5" ht="333.75" x14ac:dyDescent="0.4">
@@ -24025,10 +26650,10 @@
         <v>20</v>
       </c>
       <c r="D22" t="s">
+        <v>81</v>
+      </c>
+      <c r="E22" s="1" t="s">
         <v>82</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="23" spans="2:5" ht="236.25" x14ac:dyDescent="0.4">
@@ -24040,10 +26665,10 @@
         <v>21</v>
       </c>
       <c r="D23" t="s">
+        <v>83</v>
+      </c>
+      <c r="E23" s="1" t="s">
         <v>84</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="24" spans="2:5" ht="307.5" x14ac:dyDescent="0.4">
@@ -24055,10 +26680,10 @@
         <v>22</v>
       </c>
       <c r="D24" t="s">
+        <v>85</v>
+      </c>
+      <c r="E24" s="1" t="s">
         <v>86</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="25" spans="2:5" ht="240" x14ac:dyDescent="0.4">
@@ -24070,10 +26695,10 @@
         <v>23</v>
       </c>
       <c r="D25" t="s">
+        <v>87</v>
+      </c>
+      <c r="E25" s="1" t="s">
         <v>88</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="26" spans="2:5" ht="258.75" x14ac:dyDescent="0.4">
@@ -24085,10 +26710,10 @@
         <v>24</v>
       </c>
       <c r="D26" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="27" spans="2:5" ht="236.25" x14ac:dyDescent="0.4">
@@ -24100,10 +26725,10 @@
         <v>25</v>
       </c>
       <c r="D27" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="28" spans="2:5" ht="315" x14ac:dyDescent="0.4">
@@ -24115,10 +26740,10 @@
         <v>26</v>
       </c>
       <c r="D28" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="29" spans="2:5" ht="240" x14ac:dyDescent="0.4">
@@ -24130,10 +26755,10 @@
         <v>27</v>
       </c>
       <c r="D29" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="30" spans="2:5" ht="409.5" x14ac:dyDescent="0.4">
@@ -24145,16 +26770,46 @@
         <v>28</v>
       </c>
       <c r="D30" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
     </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="31" spans="2:5" ht="258.75" x14ac:dyDescent="0.4">
       <c r="C31">
         <f t="shared" si="0"/>
         <v>29</v>
+      </c>
+      <c r="D31" t="s">
+        <v>99</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="32" spans="2:5" ht="258.75" x14ac:dyDescent="0.4">
+      <c r="C32">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="D32" t="s">
+        <v>104</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="33" spans="3:5" ht="409.5" x14ac:dyDescent="0.4">
+      <c r="C33">
+        <f t="shared" si="0"/>
+        <v>31</v>
+      </c>
+      <c r="D33" t="s">
+        <v>109</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -24165,11 +26820,474 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49199C90-9BB8-45C0-BAA3-6AD72AA42C11}">
-  <dimension ref="B2:J19"/>
+  <dimension ref="A1:E38"/>
+  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="21.625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="33.875" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="31.375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="78.75" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="36.875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="50.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.5" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="30" x14ac:dyDescent="0.4">
+      <c r="A1" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A2" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+    </row>
+    <row r="3" spans="1:5" ht="19.5" x14ac:dyDescent="0.4">
+      <c r="A3" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="B3" s="8"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A4" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="B4" t="s">
+        <v>119</v>
+      </c>
+      <c r="C4" t="s">
+        <v>120</v>
+      </c>
+      <c r="D4" t="s">
+        <v>121</v>
+      </c>
+      <c r="E4" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="56.25" x14ac:dyDescent="0.4">
+      <c r="A5" s="5">
+        <v>1</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A6" s="4"/>
+    </row>
+    <row r="7" spans="1:5" ht="19.5" x14ac:dyDescent="0.4">
+      <c r="A7" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A8" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="B8" t="s">
+        <v>128</v>
+      </c>
+      <c r="C8" t="s">
+        <v>129</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="37.5" x14ac:dyDescent="0.4">
+      <c r="A9" s="5">
+        <v>1</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="D9" s="4"/>
+    </row>
+    <row r="10" spans="1:5" ht="37.5" x14ac:dyDescent="0.4">
+      <c r="A10" s="5">
+        <v>2</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="37.5" x14ac:dyDescent="0.4">
+      <c r="A11" s="5">
+        <v>3</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="37.5" x14ac:dyDescent="0.4">
+      <c r="A12" s="5">
+        <v>4</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="37.5" x14ac:dyDescent="0.4">
+      <c r="A13" s="5">
+        <v>5</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="37.5" x14ac:dyDescent="0.4">
+      <c r="A14" s="5">
+        <v>6</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="37.5" x14ac:dyDescent="0.4">
+      <c r="A15" s="5">
+        <v>7</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="37.5" x14ac:dyDescent="0.4">
+      <c r="A16" s="5">
+        <v>8</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="37.5" x14ac:dyDescent="0.4">
+      <c r="A17" s="5">
+        <v>9</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="37.5" x14ac:dyDescent="0.4">
+      <c r="A18" s="5">
+        <v>10</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="37.5" x14ac:dyDescent="0.4">
+      <c r="A19" s="5">
+        <v>11</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="37.5" x14ac:dyDescent="0.4">
+      <c r="A20" s="5">
+        <v>12</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A21" s="5">
+        <v>13</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="C21" s="1"/>
+      <c r="D21" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="19.5" x14ac:dyDescent="0.4">
+      <c r="A23" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="B23" s="8"/>
+      <c r="C23" s="8"/>
+      <c r="D23" s="8"/>
+      <c r="E23" s="8"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A24" t="s">
+        <v>153</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="C24" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A25" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C25" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A26" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C26" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A27" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C27" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A28" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C28" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A29" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C29" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A30" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C30" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A31" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C31" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A32" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C32" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A33" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C33" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A34" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C34" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A35" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="B35" s="4"/>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A36" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="B36" s="4"/>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A37" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B37" s="4"/>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A38" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A7:E7"/>
+    <mergeCell ref="A23:E23"/>
+  </mergeCells>
+  <phoneticPr fontId="1"/>
+  <conditionalFormatting sqref="B25:B38">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+      <formula>"〇"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D9:D21">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
+      <formula>"〇"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="3">
+    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06BEF523-B434-4C32-9B44-37C4DE1DAAF0}">
+  <dimension ref="B2:H15"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="2.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="62.375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="49.625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="78.75" bestFit="1" customWidth="1"/>
@@ -24178,245 +27296,280 @@
     <col min="9" max="9" width="21.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:8" x14ac:dyDescent="0.4">
       <c r="E2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="F2" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:8" x14ac:dyDescent="0.4">
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>94</v>
+        <v>113</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>77</v>
+        <v>112</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>95</v>
+        <v>166</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="G3" t="s">
-        <v>94</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>105</v>
-      </c>
+        <v>167</v>
+      </c>
+      <c r="H3" s="3"/>
     </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="B4">
+        <f>B3+1</f>
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>168</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>176</v>
+      </c>
       <c r="F4" t="s">
         <v>1</v>
       </c>
-      <c r="G4" t="s">
-        <v>102</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>109</v>
-      </c>
+      <c r="H4" s="3"/>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.4">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="B5">
+        <f>B4+1</f>
+        <v>3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>181</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>182</v>
+      </c>
       <c r="F5" t="s">
         <v>1</v>
       </c>
-      <c r="G5" t="s">
-        <v>107</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>110</v>
-      </c>
+      <c r="H5" s="3"/>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:8" x14ac:dyDescent="0.4">
       <c r="F6" t="s">
         <v>1</v>
       </c>
-      <c r="G6" t="s">
-        <v>108</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>112</v>
-      </c>
+      <c r="H6" s="3"/>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.4">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.4">
       <c r="F7" t="s">
         <v>1</v>
       </c>
-      <c r="G7" t="s">
-        <v>111</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="I7" t="s">
-        <v>116</v>
-      </c>
-      <c r="J7" t="s">
-        <v>1</v>
-      </c>
+      <c r="H7" s="3"/>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.4">
+    <row r="8" spans="2:8" x14ac:dyDescent="0.4">
       <c r="F8" t="s">
         <v>1</v>
       </c>
-      <c r="G8" t="s">
-        <v>111</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="I8" t="s">
-        <v>115</v>
-      </c>
-      <c r="J8" t="s">
-        <v>1</v>
-      </c>
+      <c r="H8" s="3"/>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:8" x14ac:dyDescent="0.4">
       <c r="F9" t="s">
         <v>1</v>
       </c>
-      <c r="G9" t="s">
-        <v>117</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="I9" t="s">
-        <v>122</v>
-      </c>
-      <c r="J9" t="s">
-        <v>1</v>
-      </c>
+      <c r="H9" s="3"/>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:8" x14ac:dyDescent="0.4">
       <c r="F10" t="s">
         <v>1</v>
       </c>
-      <c r="G10" t="s">
-        <v>118</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="I10" t="s">
-        <v>123</v>
-      </c>
-      <c r="J10" t="s">
-        <v>1</v>
-      </c>
+      <c r="H10" s="3"/>
     </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.4">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.4">
       <c r="F11" t="s">
         <v>1</v>
       </c>
-      <c r="G11" t="s">
-        <v>121</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="I11" t="s">
-        <v>124</v>
-      </c>
-      <c r="J11" t="s">
-        <v>1</v>
-      </c>
+      <c r="H11" s="3"/>
     </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.4">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.4">
       <c r="F12" t="s">
         <v>1</v>
       </c>
-      <c r="G12" t="s">
-        <v>129</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="I12" t="s">
-        <v>125</v>
-      </c>
-      <c r="J12" t="s">
-        <v>1</v>
-      </c>
+      <c r="H12" s="3"/>
     </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.4">
+    <row r="13" spans="2:8" x14ac:dyDescent="0.4">
       <c r="F13" t="s">
         <v>1</v>
       </c>
-      <c r="G13" t="s">
-        <v>131</v>
-      </c>
-      <c r="H13" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="I13" t="s">
-        <v>134</v>
-      </c>
+      <c r="H13" s="3"/>
     </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.4">
-      <c r="G14" t="s">
-        <v>133</v>
-      </c>
-      <c r="I14" t="s">
-        <v>135</v>
-      </c>
+    <row r="14" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="F14" t="s">
+        <v>1</v>
+      </c>
+      <c r="H14" s="3"/>
     </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.4">
-      <c r="I15" t="s">
-        <v>136</v>
-      </c>
-      <c r="J15" t="s">
+    <row r="15" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="F15" t="s">
         <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.4">
-      <c r="I16" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="17" spans="9:9" x14ac:dyDescent="0.4">
-      <c r="I17" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="18" spans="9:9" x14ac:dyDescent="0.4">
-      <c r="I18" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="19" spans="9:9" x14ac:dyDescent="0.4">
-      <c r="I19" t="s">
-        <v>140</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>
   <hyperlinks>
-    <hyperlink ref="D3" r:id="rId1" xr:uid="{519012D9-D57E-4685-BBA6-CB1C8061383A}"/>
-    <hyperlink ref="E3" r:id="rId2" xr:uid="{105F50FE-3BAA-4EAE-867D-A196B32BB119}"/>
-    <hyperlink ref="H3" r:id="rId3" xr:uid="{F9F88046-A983-43FE-A30C-07771C0C5A43}"/>
-    <hyperlink ref="F3" r:id="rId4" xr:uid="{10580E7B-8AA3-47D8-942A-F28AB2887FD5}"/>
-    <hyperlink ref="H4" r:id="rId5" xr:uid="{03BB2B03-8C36-4017-A518-CE3BC314953D}"/>
-    <hyperlink ref="H5" r:id="rId6" xr:uid="{5F2D1BB3-51D2-4792-8A97-B48004C15BAA}"/>
-    <hyperlink ref="H6" r:id="rId7" xr:uid="{1E91F52D-EDCF-444F-A15C-D01E5DA67DFC}"/>
-    <hyperlink ref="H7" r:id="rId8" xr:uid="{0D564E43-38C4-48F4-AAAB-4525354FC72F}"/>
-    <hyperlink ref="H8" r:id="rId9" xr:uid="{C0D26131-7E05-42BC-82C1-BF5A3C8CA0AA}"/>
-    <hyperlink ref="H9" r:id="rId10" xr:uid="{064DA19D-7439-463F-82FE-C95706338D47}"/>
-    <hyperlink ref="H10" r:id="rId11" xr:uid="{14228D45-42B2-48B7-925F-FA241A01441B}"/>
-    <hyperlink ref="H11" r:id="rId12" xr:uid="{367E638D-234E-4EDB-AEF7-C988D3EC6D19}"/>
-    <hyperlink ref="H12" r:id="rId13" xr:uid="{1F218158-2EA3-4B0C-BF90-D126C575D2B6}"/>
-    <hyperlink ref="H13" r:id="rId14" xr:uid="{4ED2049A-D59E-4607-9BBE-3F4210108A82}"/>
+    <hyperlink ref="D3" r:id="rId1" xr:uid="{D7A01C7E-D543-411B-B28A-F0C4B2147C84}"/>
+    <hyperlink ref="E3" r:id="rId2" xr:uid="{D67DD94E-D8FA-4E8C-ACF1-A6C812EED56C}"/>
+    <hyperlink ref="F3" r:id="rId3" xr:uid="{5768FE47-DF4C-4128-9AF7-CA0B6A568B07}"/>
+    <hyperlink ref="D4" r:id="rId4" xr:uid="{9BCEC014-F93D-47D8-9FAE-4A1DA92B19D9}"/>
+    <hyperlink ref="E4" r:id="rId5" xr:uid="{C0B5B1BE-153B-420B-B3F4-693F65193819}"/>
+    <hyperlink ref="D5" r:id="rId6" xr:uid="{3AC3A764-8357-466F-9958-56623369F1E2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4ADA3461-3FC5-4E21-A085-8E75E91C0BA9}">
+  <dimension ref="B2:G7"/>
+  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="2" max="2" width="2.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="77.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="48.375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="77.375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="E2" t="s">
+        <v>93</v>
+      </c>
+      <c r="F2" t="s">
+        <v>94</v>
+      </c>
+      <c r="G2" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>174</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="G3" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="B4">
+        <f>B3+1</f>
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>178</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="F4" t="s">
+        <v>1</v>
+      </c>
+      <c r="G4" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="B5">
+        <f>B4+1</f>
+        <v>3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>184</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="F5" t="s">
+        <v>1</v>
+      </c>
+      <c r="G5" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="B6">
+        <f>B5+1</f>
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>187</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="F6" t="s">
+        <v>1</v>
+      </c>
+      <c r="G6" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="B7">
+        <f>B6+1</f>
+        <v>5</v>
+      </c>
+      <c r="C7" t="s">
+        <v>191</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="F7" t="s">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <hyperlinks>
+    <hyperlink ref="D3" r:id="rId1" xr:uid="{137CE8D7-B230-441C-A546-6C7A3A25674F}"/>
+    <hyperlink ref="E3" r:id="rId2" xr:uid="{CF32CD14-EA3C-433E-88FE-13FB85693333}"/>
+    <hyperlink ref="F3" r:id="rId3" xr:uid="{027C4A4C-AC0D-4CF8-8730-225F983CA595}"/>
+    <hyperlink ref="D4" r:id="rId4" xr:uid="{9E41268E-7F13-4BD7-8F0B-64F329BDBE7D}"/>
+    <hyperlink ref="E4" r:id="rId5" xr:uid="{96172731-C12D-4AED-B7A7-9283CCA8E687}"/>
+    <hyperlink ref="D5" r:id="rId6" xr:uid="{05CDA43B-635F-4E60-9722-DE1AFB891F50}"/>
+    <hyperlink ref="E5" r:id="rId7" xr:uid="{242195AF-69F3-4D62-89CC-02A48B20D497}"/>
+    <hyperlink ref="D6" r:id="rId8" xr:uid="{93488C18-17D5-4AA3-BDD3-DF6E45591AD2}"/>
+    <hyperlink ref="E6" r:id="rId9" xr:uid="{7131FFA0-BABE-4EB1-A5BC-2EF10BF8B3E1}"/>
+    <hyperlink ref="D7" r:id="rId10" xr:uid="{F2481D20-8F5F-448C-B8AF-2B038779C9B1}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FFF1E46-B8F1-4111-9292-CB57C462E366}">
   <dimension ref="A2:F6"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
@@ -24520,7 +27673,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3130DC33-D7DC-49CA-BAC6-4FF425438F8A}">
   <dimension ref="A2:D3"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
@@ -24558,7 +27711,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C864D64-BD4E-47C2-98A7-786282D674DD}">
   <dimension ref="B3:D3"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
@@ -24573,10 +27726,10 @@
         <v>1</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>126</v>
+        <v>101</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>127</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>

</xml_diff>